<commit_message>
Se agrega codigo para linea de 5mm, altura de cámara 15cm, tolerancia 5%
</commit_message>
<xml_diff>
--- a/Informes/Gantt Vehículo Autónomo.xlsx
+++ b/Informes/Gantt Vehículo Autónomo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a31f0271d0b8797b/Desktop/Proyecto Ingenieria/INFORMES/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a31f0271d0b8797b/Desktop/Proyecto Ingenieria/2026_2C_PF_VEHICULO-AUTONOMO-MARCADO-DE-LAYOUTS_ESPINOLA-SULLCA-main/Informes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="646" documentId="8_{A2B61D2F-08BD-40F5-ACC5-C73775A42AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9ABC49D0-F1D8-47A4-B507-E0F67FD6380F}"/>
+  <xr:revisionPtr revIDLastSave="654" documentId="8_{A2B61D2F-08BD-40F5-ACC5-C73775A42AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6F830BB-8838-4375-B993-848ABF3B6A14}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1692,14 +1692,39 @@
     <xf numFmtId="0" fontId="0" fillId="20" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="21" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="21" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1716,42 +1741,17 @@
     <xf numFmtId="167" fontId="15" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="18" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="21" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="21" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -1894,6 +1894,25 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1990,25 +2009,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="_-[$$-409]* #,##0_ ;_-[$$-409]* \-#,##0\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border>
@@ -2208,7 +2208,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7B046895-9170-4AC6-8C65-BF0F2537217B}" name="Tabla3" displayName="Tabla3" ref="C2:F23" totalsRowShown="0" headerRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7B046895-9170-4AC6-8C65-BF0F2537217B}" name="Tabla3" displayName="Tabla3" ref="C2:F23" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="C2:F23" xr:uid="{7B046895-9170-4AC6-8C65-BF0F2537217B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2216,10 +2216,10 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{677FC96E-7F25-4A06-87E3-922FDD41B915}" name="Tarea" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{58277187-363E-428B-A83B-BC14DB987A6B}" name="Horas estimadas" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{488EC91C-90C1-4FC4-A305-62832539CD69}" name="Horas reales" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{C0DE1A19-3FEF-4849-899B-C98251D2724D}" name="Diferencia" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{677FC96E-7F25-4A06-87E3-922FDD41B915}" name="Tarea" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{58277187-363E-428B-A83B-BC14DB987A6B}" name="Horas estimadas" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{488EC91C-90C1-4FC4-A305-62832539CD69}" name="Horas reales" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{C0DE1A19-3FEF-4849-899B-C98251D2724D}" name="Diferencia" dataDxfId="15">
       <calculatedColumnFormula>Tabla3[[#This Row],[Horas reales]]-Tabla3[[#This Row],[Horas estimadas]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2238,12 +2238,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{45ACA5F6-477D-42B6-B421-4AEE018B4E81}" name="Nombre" totalsRowLabel="Total" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{CDC2B791-5EFB-4C87-AAD3-192DBB5C19D6}" name="Descripción" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{45ACA5F6-477D-42B6-B421-4AEE018B4E81}" name="Nombre" totalsRowLabel="Total" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{CDC2B791-5EFB-4C87-AAD3-192DBB5C19D6}" name="Descripción" dataDxfId="13"/>
     <tableColumn id="3" xr3:uid="{95A5BD7C-444C-4C6D-BE74-E16B3FFFEE8E}" name="Cantidad"/>
     <tableColumn id="4" xr3:uid="{FF7F68A1-0DEA-4B69-8384-B1FE22AD9958}" name="Proveedor"/>
-    <tableColumn id="5" xr3:uid="{63F8E491-A0B5-4A72-A3FF-8221530F268B}" name="Precio unitario" totalsRowLabel=" $ARS " dataDxfId="17" totalsRowDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{1E275AE4-1059-4BEF-B3F7-9BB27037631B}" name="Total" totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{63F8E491-A0B5-4A72-A3FF-8221530F268B}" name="Precio unitario" totalsRowLabel=" $ARS " dataDxfId="12" totalsRowDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{1E275AE4-1059-4BEF-B3F7-9BB27037631B}" name="Total" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2499,28 +2499,28 @@
       <c r="G1" s="12"/>
       <c r="H1" s="13"/>
       <c r="J1" s="1"/>
-      <c r="K1" s="176" t="s">
+      <c r="K1" s="185" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
-      <c r="Q1" s="177"/>
+      <c r="L1" s="186"/>
+      <c r="M1" s="186"/>
+      <c r="N1" s="186"/>
+      <c r="O1" s="186"/>
+      <c r="P1" s="186"/>
+      <c r="Q1" s="186"/>
       <c r="R1" s="16"/>
-      <c r="S1" s="178">
+      <c r="S1" s="187">
         <v>46244</v>
       </c>
-      <c r="T1" s="179"/>
-      <c r="U1" s="179"/>
-      <c r="V1" s="179"/>
-      <c r="W1" s="179"/>
-      <c r="X1" s="179"/>
-      <c r="Y1" s="179"/>
-      <c r="Z1" s="179"/>
-      <c r="AA1" s="179"/>
-      <c r="AB1" s="179"/>
+      <c r="T1" s="188"/>
+      <c r="U1" s="188"/>
+      <c r="V1" s="188"/>
+      <c r="W1" s="188"/>
+      <c r="X1" s="188"/>
+      <c r="Y1" s="188"/>
+      <c r="Z1" s="188"/>
+      <c r="AA1" s="188"/>
+      <c r="AB1" s="188"/>
     </row>
     <row r="2" spans="1:66" ht="30" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A2" s="71" t="s">
@@ -2535,28 +2535,28 @@
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
       <c r="H2" s="14"/>
-      <c r="K2" s="176" t="s">
+      <c r="K2" s="185" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="177"/>
-      <c r="M2" s="177"/>
-      <c r="N2" s="177"/>
-      <c r="O2" s="177"/>
-      <c r="P2" s="177"/>
-      <c r="Q2" s="177"/>
+      <c r="L2" s="186"/>
+      <c r="M2" s="186"/>
+      <c r="N2" s="186"/>
+      <c r="O2" s="186"/>
+      <c r="P2" s="186"/>
+      <c r="Q2" s="186"/>
       <c r="R2" s="16"/>
-      <c r="S2" s="180">
-        <v>2</v>
-      </c>
-      <c r="T2" s="181"/>
-      <c r="U2" s="181"/>
-      <c r="V2" s="181"/>
-      <c r="W2" s="181"/>
-      <c r="X2" s="181"/>
-      <c r="Y2" s="181"/>
-      <c r="Z2" s="181"/>
-      <c r="AA2" s="181"/>
-      <c r="AB2" s="181"/>
+      <c r="S2" s="189">
+        <v>1</v>
+      </c>
+      <c r="T2" s="190"/>
+      <c r="U2" s="190"/>
+      <c r="V2" s="190"/>
+      <c r="W2" s="190"/>
+      <c r="X2" s="190"/>
+      <c r="Y2" s="190"/>
+      <c r="Z2" s="190"/>
+      <c r="AA2" s="190"/>
+      <c r="AB2" s="190"/>
     </row>
     <row r="3" spans="1:66" s="18" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
@@ -2572,346 +2572,346 @@
       <c r="E4" s="22"/>
       <c r="F4" s="22"/>
       <c r="G4" s="22"/>
-      <c r="K4" s="182">
+      <c r="K4" s="191">
         <f>K5</f>
+        <v>46244</v>
+      </c>
+      <c r="L4" s="175"/>
+      <c r="M4" s="175"/>
+      <c r="N4" s="175"/>
+      <c r="O4" s="175"/>
+      <c r="P4" s="175"/>
+      <c r="Q4" s="175"/>
+      <c r="R4" s="175">
+        <f>R5</f>
         <v>46251</v>
       </c>
-      <c r="L4" s="183"/>
-      <c r="M4" s="183"/>
-      <c r="N4" s="183"/>
-      <c r="O4" s="183"/>
-      <c r="P4" s="183"/>
-      <c r="Q4" s="183"/>
-      <c r="R4" s="183">
-        <f>R5</f>
+      <c r="S4" s="175"/>
+      <c r="T4" s="175"/>
+      <c r="U4" s="175"/>
+      <c r="V4" s="175"/>
+      <c r="W4" s="175"/>
+      <c r="X4" s="175"/>
+      <c r="Y4" s="175">
+        <f>Y5</f>
         <v>46258</v>
       </c>
-      <c r="S4" s="183"/>
-      <c r="T4" s="183"/>
-      <c r="U4" s="183"/>
-      <c r="V4" s="183"/>
-      <c r="W4" s="183"/>
-      <c r="X4" s="183"/>
-      <c r="Y4" s="183">
-        <f>Y5</f>
+      <c r="Z4" s="175"/>
+      <c r="AA4" s="175"/>
+      <c r="AB4" s="175"/>
+      <c r="AC4" s="175"/>
+      <c r="AD4" s="175"/>
+      <c r="AE4" s="175"/>
+      <c r="AF4" s="175">
+        <f>AF5</f>
         <v>46265</v>
       </c>
-      <c r="Z4" s="183"/>
-      <c r="AA4" s="183"/>
-      <c r="AB4" s="183"/>
-      <c r="AC4" s="183"/>
-      <c r="AD4" s="183"/>
-      <c r="AE4" s="183"/>
-      <c r="AF4" s="183">
-        <f>AF5</f>
+      <c r="AG4" s="175"/>
+      <c r="AH4" s="175"/>
+      <c r="AI4" s="175"/>
+      <c r="AJ4" s="175"/>
+      <c r="AK4" s="175"/>
+      <c r="AL4" s="175"/>
+      <c r="AM4" s="175">
+        <f>AM5</f>
         <v>46272</v>
       </c>
-      <c r="AG4" s="183"/>
-      <c r="AH4" s="183"/>
-      <c r="AI4" s="183"/>
-      <c r="AJ4" s="183"/>
-      <c r="AK4" s="183"/>
-      <c r="AL4" s="183"/>
-      <c r="AM4" s="183">
-        <f>AM5</f>
+      <c r="AN4" s="175"/>
+      <c r="AO4" s="175"/>
+      <c r="AP4" s="175"/>
+      <c r="AQ4" s="175"/>
+      <c r="AR4" s="175"/>
+      <c r="AS4" s="175"/>
+      <c r="AT4" s="175">
+        <f>AT5</f>
         <v>46279</v>
       </c>
-      <c r="AN4" s="183"/>
-      <c r="AO4" s="183"/>
-      <c r="AP4" s="183"/>
-      <c r="AQ4" s="183"/>
-      <c r="AR4" s="183"/>
-      <c r="AS4" s="183"/>
-      <c r="AT4" s="183">
-        <f>AT5</f>
+      <c r="AU4" s="175"/>
+      <c r="AV4" s="175"/>
+      <c r="AW4" s="175"/>
+      <c r="AX4" s="175"/>
+      <c r="AY4" s="175"/>
+      <c r="AZ4" s="175"/>
+      <c r="BA4" s="175">
+        <f>BA5</f>
         <v>46286</v>
       </c>
-      <c r="AU4" s="183"/>
-      <c r="AV4" s="183"/>
-      <c r="AW4" s="183"/>
-      <c r="AX4" s="183"/>
-      <c r="AY4" s="183"/>
-      <c r="AZ4" s="183"/>
-      <c r="BA4" s="183">
-        <f>BA5</f>
+      <c r="BB4" s="175"/>
+      <c r="BC4" s="175"/>
+      <c r="BD4" s="175"/>
+      <c r="BE4" s="175"/>
+      <c r="BF4" s="175"/>
+      <c r="BG4" s="175"/>
+      <c r="BH4" s="175">
+        <f>BH5</f>
         <v>46293</v>
       </c>
-      <c r="BB4" s="183"/>
-      <c r="BC4" s="183"/>
-      <c r="BD4" s="183"/>
-      <c r="BE4" s="183"/>
-      <c r="BF4" s="183"/>
-      <c r="BG4" s="183"/>
-      <c r="BH4" s="183">
-        <f>BH5</f>
-        <v>46300</v>
-      </c>
-      <c r="BI4" s="183"/>
-      <c r="BJ4" s="183"/>
-      <c r="BK4" s="183"/>
-      <c r="BL4" s="183"/>
-      <c r="BM4" s="183"/>
-      <c r="BN4" s="184"/>
+      <c r="BI4" s="175"/>
+      <c r="BJ4" s="175"/>
+      <c r="BK4" s="175"/>
+      <c r="BL4" s="175"/>
+      <c r="BM4" s="175"/>
+      <c r="BN4" s="176"/>
     </row>
     <row r="5" spans="1:66" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="185" t="s">
+      <c r="A5" s="177" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="187" t="s">
+      <c r="B5" s="179" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="189" t="s">
+      <c r="C5" s="181" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="189" t="s">
+      <c r="D5" s="181" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="189" t="s">
+      <c r="E5" s="181" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="189" t="s">
+      <c r="F5" s="181" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="194" t="s">
+      <c r="G5" s="183" t="s">
         <v>97</v>
       </c>
-      <c r="H5" s="194" t="s">
+      <c r="H5" s="183" t="s">
         <v>98</v>
       </c>
       <c r="K5" s="23">
         <f>Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
-        <v>46251</v>
+        <v>46244</v>
       </c>
       <c r="L5" s="23">
         <f>K5+1</f>
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="M5" s="23">
         <f t="shared" ref="M5:AZ5" si="0">L5+1</f>
-        <v>46253</v>
+        <v>46246</v>
       </c>
       <c r="N5" s="23">
         <f t="shared" si="0"/>
-        <v>46254</v>
+        <v>46247</v>
       </c>
       <c r="O5" s="23">
         <f t="shared" si="0"/>
-        <v>46255</v>
+        <v>46248</v>
       </c>
       <c r="P5" s="23">
         <f t="shared" si="0"/>
-        <v>46256</v>
+        <v>46249</v>
       </c>
       <c r="Q5" s="24">
         <f t="shared" si="0"/>
-        <v>46257</v>
+        <v>46250</v>
       </c>
       <c r="R5" s="25">
         <f>Q5+1</f>
-        <v>46258</v>
+        <v>46251</v>
       </c>
       <c r="S5" s="23">
         <f>R5+1</f>
-        <v>46259</v>
+        <v>46252</v>
       </c>
       <c r="T5" s="23">
         <f t="shared" si="0"/>
-        <v>46260</v>
+        <v>46253</v>
       </c>
       <c r="U5" s="23">
         <f t="shared" si="0"/>
-        <v>46261</v>
+        <v>46254</v>
       </c>
       <c r="V5" s="23">
         <f t="shared" si="0"/>
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="W5" s="23">
         <f t="shared" si="0"/>
-        <v>46263</v>
+        <v>46256</v>
       </c>
       <c r="X5" s="24">
         <f t="shared" si="0"/>
-        <v>46264</v>
+        <v>46257</v>
       </c>
       <c r="Y5" s="25">
         <f>X5+1</f>
-        <v>46265</v>
+        <v>46258</v>
       </c>
       <c r="Z5" s="23">
         <f>Y5+1</f>
-        <v>46266</v>
+        <v>46259</v>
       </c>
       <c r="AA5" s="23">
         <f t="shared" si="0"/>
-        <v>46267</v>
+        <v>46260</v>
       </c>
       <c r="AB5" s="23">
         <f t="shared" si="0"/>
-        <v>46268</v>
+        <v>46261</v>
       </c>
       <c r="AC5" s="23">
         <f t="shared" si="0"/>
-        <v>46269</v>
+        <v>46262</v>
       </c>
       <c r="AD5" s="23">
         <f t="shared" si="0"/>
-        <v>46270</v>
+        <v>46263</v>
       </c>
       <c r="AE5" s="24">
         <f t="shared" si="0"/>
-        <v>46271</v>
+        <v>46264</v>
       </c>
       <c r="AF5" s="25">
         <f>AE5+1</f>
-        <v>46272</v>
+        <v>46265</v>
       </c>
       <c r="AG5" s="23">
         <f>AF5+1</f>
-        <v>46273</v>
+        <v>46266</v>
       </c>
       <c r="AH5" s="23">
         <f t="shared" si="0"/>
-        <v>46274</v>
+        <v>46267</v>
       </c>
       <c r="AI5" s="23">
         <f t="shared" si="0"/>
-        <v>46275</v>
+        <v>46268</v>
       </c>
       <c r="AJ5" s="23">
         <f t="shared" si="0"/>
-        <v>46276</v>
+        <v>46269</v>
       </c>
       <c r="AK5" s="23">
         <f t="shared" si="0"/>
-        <v>46277</v>
+        <v>46270</v>
       </c>
       <c r="AL5" s="24">
         <f t="shared" si="0"/>
-        <v>46278</v>
+        <v>46271</v>
       </c>
       <c r="AM5" s="25">
         <f>AL5+1</f>
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="AN5" s="23">
         <f>AM5+1</f>
-        <v>46280</v>
+        <v>46273</v>
       </c>
       <c r="AO5" s="23">
         <f t="shared" si="0"/>
-        <v>46281</v>
+        <v>46274</v>
       </c>
       <c r="AP5" s="23">
         <f t="shared" si="0"/>
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="AQ5" s="23">
         <f t="shared" si="0"/>
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="AR5" s="23">
         <f t="shared" si="0"/>
-        <v>46284</v>
+        <v>46277</v>
       </c>
       <c r="AS5" s="24">
         <f t="shared" si="0"/>
-        <v>46285</v>
+        <v>46278</v>
       </c>
       <c r="AT5" s="25">
         <f>AS5+1</f>
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="AU5" s="23">
         <f>AT5+1</f>
-        <v>46287</v>
+        <v>46280</v>
       </c>
       <c r="AV5" s="23">
         <f t="shared" si="0"/>
-        <v>46288</v>
+        <v>46281</v>
       </c>
       <c r="AW5" s="23">
         <f t="shared" si="0"/>
-        <v>46289</v>
+        <v>46282</v>
       </c>
       <c r="AX5" s="23">
         <f t="shared" si="0"/>
-        <v>46290</v>
+        <v>46283</v>
       </c>
       <c r="AY5" s="23">
         <f t="shared" si="0"/>
-        <v>46291</v>
+        <v>46284</v>
       </c>
       <c r="AZ5" s="24">
         <f t="shared" si="0"/>
-        <v>46292</v>
+        <v>46285</v>
       </c>
       <c r="BA5" s="25">
         <f>AZ5+1</f>
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="BB5" s="23">
         <f>BA5+1</f>
-        <v>46294</v>
+        <v>46287</v>
       </c>
       <c r="BC5" s="23">
         <f t="shared" ref="BC5:BG5" si="1">BB5+1</f>
-        <v>46295</v>
+        <v>46288</v>
       </c>
       <c r="BD5" s="23">
         <f t="shared" si="1"/>
-        <v>46296</v>
+        <v>46289</v>
       </c>
       <c r="BE5" s="23">
         <f t="shared" si="1"/>
-        <v>46297</v>
+        <v>46290</v>
       </c>
       <c r="BF5" s="23">
         <f t="shared" si="1"/>
-        <v>46298</v>
+        <v>46291</v>
       </c>
       <c r="BG5" s="24">
         <f t="shared" si="1"/>
-        <v>46299</v>
+        <v>46292</v>
       </c>
       <c r="BH5" s="25">
         <f>BG5+1</f>
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="BI5" s="23">
         <f>BH5+1</f>
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="BJ5" s="23">
         <f t="shared" ref="BJ5:BN5" si="2">BI5+1</f>
-        <v>46302</v>
+        <v>46295</v>
       </c>
       <c r="BK5" s="23">
         <f t="shared" si="2"/>
-        <v>46303</v>
+        <v>46296</v>
       </c>
       <c r="BL5" s="23">
         <f t="shared" si="2"/>
-        <v>46304</v>
+        <v>46297</v>
       </c>
       <c r="BM5" s="23">
         <f t="shared" si="2"/>
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="BN5" s="23">
         <f t="shared" si="2"/>
-        <v>46306</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="6" spans="1:66" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="186"/>
-      <c r="B6" s="188"/>
-      <c r="C6" s="188"/>
-      <c r="D6" s="188"/>
-      <c r="E6" s="190"/>
-      <c r="F6" s="188"/>
-      <c r="G6" s="195"/>
-      <c r="H6" s="195"/>
+      <c r="A6" s="178"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="180"/>
+      <c r="D6" s="180"/>
+      <c r="E6" s="182"/>
+      <c r="F6" s="180"/>
+      <c r="G6" s="184"/>
+      <c r="H6" s="184"/>
       <c r="K6" s="26" t="str">
         <f t="shared" ref="K6:BN6" si="3">LEFT(TEXT(K5,"ddd"),1)</f>
         <v>l</v>
@@ -3578,7 +3578,7 @@
       <c r="E13" s="89">
         <v>40</v>
       </c>
-      <c r="F13" s="89">
+      <c r="F13" s="77">
         <f>D13+E13</f>
         <v>46306</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="102">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="D14" s="103">
         <v>46265</v>
@@ -3674,7 +3674,7 @@
         <v>12</v>
       </c>
       <c r="H14" s="104">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="5"/>
@@ -4066,10 +4066,10 @@
         <f>D19+E19</f>
         <v>46258</v>
       </c>
-      <c r="G19" s="192">
+      <c r="G19" s="173">
         <v>4</v>
       </c>
-      <c r="H19" s="192">
+      <c r="H19" s="173">
         <v>4</v>
       </c>
       <c r="I19" s="9"/>
@@ -4149,8 +4149,8 @@
         <f>D20+E20</f>
         <v>46293</v>
       </c>
-      <c r="G20" s="193"/>
-      <c r="H20" s="193"/>
+      <c r="G20" s="174"/>
+      <c r="H20" s="174"/>
       <c r="I20" s="9"/>
       <c r="J20" s="5"/>
       <c r="K20" s="59"/>
@@ -5238,6 +5238,13 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="K1:Q1"/>
+    <mergeCell ref="S1:AB1"/>
+    <mergeCell ref="K2:Q2"/>
+    <mergeCell ref="S2:AB2"/>
+    <mergeCell ref="K4:Q4"/>
+    <mergeCell ref="R4:X4"/>
+    <mergeCell ref="Y4:AE4"/>
     <mergeCell ref="BA4:BG4"/>
     <mergeCell ref="BH4:BN4"/>
     <mergeCell ref="A5:A6"/>
@@ -5251,13 +5258,6 @@
     <mergeCell ref="AT4:AZ4"/>
     <mergeCell ref="G5:G6"/>
     <mergeCell ref="H5:H6"/>
-    <mergeCell ref="K1:Q1"/>
-    <mergeCell ref="S1:AB1"/>
-    <mergeCell ref="K2:Q2"/>
-    <mergeCell ref="S2:AB2"/>
-    <mergeCell ref="K4:Q4"/>
-    <mergeCell ref="R4:X4"/>
-    <mergeCell ref="Y4:AE4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C33">
     <cfRule type="dataBar" priority="8">
@@ -5310,7 +5310,7 @@
       <formula>AND(task_end&gt;=K$5,task_start&lt;L$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Display Week" prompt="Changing this number will scroll the Gantt Chart view." sqref="S2" xr:uid="{5055D4DC-4AC9-4908-8988-4E07AB8DE9B0}">
       <formula1>1</formula1>
     </dataValidation>
@@ -5376,7 +5376,7 @@
       </c>
     </row>
     <row r="3" spans="2:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="191" t="s">
+      <c r="B3" s="192" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="151" t="s">
@@ -5390,7 +5390,7 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="191"/>
+      <c r="B4" s="192"/>
       <c r="C4" s="149" t="s">
         <v>43</v>
       </c>
@@ -5402,7 +5402,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="191"/>
+      <c r="B5" s="192"/>
       <c r="C5" s="149" t="s">
         <v>44</v>
       </c>
@@ -5414,7 +5414,7 @@
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="191"/>
+      <c r="B6" s="192"/>
       <c r="C6" s="149" t="s">
         <v>45</v>
       </c>
@@ -5426,7 +5426,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="191"/>
+      <c r="B7" s="192"/>
       <c r="C7" s="149"/>
       <c r="D7" s="149"/>
       <c r="E7" s="149"/>
@@ -5436,7 +5436,7 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="191"/>
+      <c r="B8" s="192"/>
       <c r="C8" s="149"/>
       <c r="D8" s="149"/>
       <c r="E8" s="149"/>
@@ -5446,7 +5446,7 @@
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="191"/>
+      <c r="B9" s="192"/>
       <c r="C9" s="149"/>
       <c r="D9" s="149"/>
       <c r="E9" s="149"/>
@@ -5456,7 +5456,7 @@
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="191"/>
+      <c r="B10" s="192"/>
       <c r="C10" s="149"/>
       <c r="D10" s="149"/>
       <c r="E10" s="149"/>
@@ -5466,7 +5466,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="191"/>
+      <c r="B11" s="192"/>
       <c r="C11" s="149"/>
       <c r="D11" s="149"/>
       <c r="E11" s="149"/>
@@ -5476,7 +5476,7 @@
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="191"/>
+      <c r="B12" s="192"/>
       <c r="C12" s="149"/>
       <c r="D12" s="149"/>
       <c r="E12" s="149"/>
@@ -5486,7 +5486,7 @@
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="191" t="s">
+      <c r="B13" s="192" t="s">
         <v>46</v>
       </c>
       <c r="C13" s="149"/>
@@ -5498,7 +5498,7 @@
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="191"/>
+      <c r="B14" s="192"/>
       <c r="C14" s="149"/>
       <c r="D14" s="149"/>
       <c r="E14" s="149"/>
@@ -5508,7 +5508,7 @@
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="191"/>
+      <c r="B15" s="192"/>
       <c r="C15" s="149"/>
       <c r="D15" s="149"/>
       <c r="E15" s="149"/>
@@ -5518,7 +5518,7 @@
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="191"/>
+      <c r="B16" s="192"/>
       <c r="C16" s="149"/>
       <c r="D16" s="149"/>
       <c r="E16" s="149"/>
@@ -5528,7 +5528,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="191"/>
+      <c r="B17" s="192"/>
       <c r="C17" s="149"/>
       <c r="D17" s="149"/>
       <c r="E17" s="149"/>
@@ -5538,7 +5538,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="191"/>
+      <c r="B18" s="192"/>
       <c r="C18" s="149"/>
       <c r="D18" s="149"/>
       <c r="E18" s="149"/>
@@ -5548,7 +5548,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="191"/>
+      <c r="B19" s="192"/>
       <c r="C19" s="149"/>
       <c r="D19" s="149"/>
       <c r="E19" s="149"/>
@@ -5558,7 +5558,7 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="191"/>
+      <c r="B20" s="192"/>
       <c r="C20" s="149"/>
       <c r="D20" s="149"/>
       <c r="E20" s="149"/>
@@ -5568,7 +5568,7 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="191"/>
+      <c r="B21" s="192"/>
       <c r="C21" s="149"/>
       <c r="D21" s="149"/>
       <c r="E21" s="149"/>
@@ -5578,7 +5578,7 @@
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="191"/>
+      <c r="B22" s="192"/>
       <c r="C22" s="149"/>
       <c r="D22" s="149"/>
       <c r="E22" s="149"/>
@@ -5588,7 +5588,7 @@
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="191"/>
+      <c r="B23" s="192"/>
       <c r="C23" s="149"/>
       <c r="D23" s="149"/>
       <c r="E23" s="149"/>
@@ -5623,14 +5623,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B1" s="173" t="s">
+      <c r="B1" s="193" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="175"/>
+      <c r="C1" s="194"/>
+      <c r="D1" s="194"/>
+      <c r="E1" s="194"/>
+      <c r="F1" s="194"/>
+      <c r="G1" s="195"/>
     </row>
     <row r="2" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
@@ -5817,12 +5817,12 @@
         <f>Tabla1[[#This Row],[Precio unitario]]*Tabla1[[#This Row],[Cantidad]]</f>
         <v>13000</v>
       </c>
-      <c r="L10" s="173"/>
-      <c r="M10" s="174"/>
-      <c r="N10" s="174"/>
-      <c r="O10" s="174"/>
-      <c r="P10" s="174"/>
-      <c r="Q10" s="175"/>
+      <c r="L10" s="193"/>
+      <c r="M10" s="194"/>
+      <c r="N10" s="194"/>
+      <c r="O10" s="194"/>
+      <c r="P10" s="194"/>
+      <c r="Q10" s="195"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B11" s="145" t="s">
@@ -6207,6 +6207,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -6518,36 +6547,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A09426A3-87E9-4865-8A6C-3456B026AE03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6568,26 +6588,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>